<commit_message>
Adiciona 6 docs novos de AASP_Andamento-Processuais ao indice (260 -> 266)
Localizados via search_files na pasta 04_registros/AASP_Andamento-Processuais
(IDs atuais do Drive); os 20 itens ja mapeados seguem com os mesmos IDs.

- MQ-AASPAP01-001_Definicao-de-Metas-de-Qualidade.docx
- ATA-AASPAP01-002_Ata-de-Acompanhamento-Fase-1.docx
- ATA-AASPAP01-003_Ata-de-Acompanhamento-Fase-2.docx
- ATA-AASPAP01-004_Ata-de-Acompanhamento-Fase-3.docx
- ATA-AASPAP01-005_Ata-de-Acompanhamento-Fase-4.docx
- REV-AASPAP01-002_Registro-de-Revisao-por-Pares-por-Entrega.docx

Mapa: 266 arquivos, 228 .docx. Sem ids/documentos duplicados.

https://claude.ai/code/session_01Le3EZ8QjyEACMRtgYDCzkN
</commit_message>
<xml_diff>
--- a/MAPA-DRIVE_Indice-de-Links.xlsx
+++ b/MAPA-DRIVE_Indice-de-Links.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Mapa de Links Drive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mapa de Links Drive'!$A$1:$D$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mapa de Links Drive'!$A$1:$D$267</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D261"/>
+  <dimension ref="A1:D267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>CR-AASPAP01-001_Change-Request.docx</t>
+          <t>ATA-AASPAP01-002_Ata-de-Acompanhamento-Fase-1.docx</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1p94Xtd_QSXghPgdDQiaj9m8JoArrHree/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1o5hMgR4SdNrl2fakLB59tI0JOtZWxlwD/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CR-AASPAP01-002_Change-Request.docx</t>
+          <t>ATA-AASPAP01-003_Ata-de-Acompanhamento-Fase-2.docx</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1e495VArI_U_3TMW7KQc0p3GfqUiAek4a/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1L5XOH48-U99-Y1mdKjuNV_UCY_bZCxJo/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>GCO-AASPAP01-001_Registro-de-Configuracao.docx</t>
+          <t>ATA-AASPAP01-004_Ata-de-Acompanhamento-Fase-3.docx</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Rl6GXnN1H9mRl0V6bSYw9Pl_D-0THH_O/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1KTLJHZC0eTeQ429HoZqPT5SoF27e_aMw/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>GDE-AASPAP01-001_Registro-de-Analise-de-Decisao.docx</t>
+          <t>ATA-AASPAP01-005_Ata-de-Acompanhamento-Fase-4.docx</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1sDGfP0m6WdyKS4MYzHLLZNNQCyus0xJw/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1U8rsYKXxRluVYXT1UNe3h5RlWmJGvS6-/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3033,17 +3033,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx</t>
+          <t>CR-AASPAP01-001_Change-Request.docx</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ZB2yOn7Pt1eviyaL1-XMCaiamiCql6gz/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1p94Xtd_QSXghPgdDQiaj9m8JoArrHree/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3055,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>GQA-AASPAP01-001_Registro-de-GQA.docx</t>
+          <t>CR-AASPAP01-002_Change-Request.docx</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19WE56UNWv-aVGiPL24PzStXvX1NuplXF/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1e495VArI_U_3TMW7KQc0p3GfqUiAek4a/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>ITP-AASPAP01-001_Estrategia-de-Integracao.docx</t>
+          <t>GCO-AASPAP01-001_Registro-de-Configuracao.docx</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1cSlw8Kqi3fPboNG2KDMoRuWYLii5s1Qm/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Rl6GXnN1H9mRl0V6bSYw9Pl_D-0THH_O/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>MED-AASPAP01-001_Registro-de-Medicao.docx</t>
+          <t>GDE-AASPAP01-001_Registro-de-Analise-de-Decisao.docx</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17jDdprZJdXPr-muQAYnQNXoMNU1VOSAV/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1sDGfP0m6WdyKS4MYzHLLZNNQCyus0xJw/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3121,17 +3121,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PCP-AASPAP01-001_Documento-de-Design.docx</t>
+          <t>GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1MkxkyhMa5O4d9ee1JVYHNZV59BxiHU3m/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ZB2yOn7Pt1eviyaL1-XMCaiamiCql6gz/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PLA-AASPAP01-001_Plano-de-Projeto.docx</t>
+          <t>GQA-AASPAP01-001_Registro-de-GQA.docx</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1D7tchEQKaqeZMZ2vNNa0wgnXevI-Br8H/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/19WE56UNWv-aVGiPL24PzStXvX1NuplXF/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>RAC-AASPAP01-001_Relatorio-de-Acompanhamento.docx</t>
+          <t>ITP-AASPAP01-001_Estrategia-de-Integracao.docx</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/155bBfagbpaZdKxRSqXQzkmZSQkmCHNt0/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1cSlw8Kqi3fPboNG2KDMoRuWYLii5s1Qm/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>RASTR-AASPAP01-001_Matriz-de-Rastreabilidade.docx</t>
+          <t>MED-AASPAP01-001_Registro-de-Medicao.docx</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nqVdGrDD5CJ_3zPB3IehiBEhuDKSxZlS/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17jDdprZJdXPr-muQAYnQNXoMNU1VOSAV/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>REL-VV-AASPAP01-001_Relatorio-de-Execucao-de-Testes.docx</t>
+          <t>MQ-AASPAP01-001_Definicao-de-Metas-de-Qualidade.docx</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1TzIWFlAfEpqwWO0JIF3DACKPzPgC2sPV/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1xsxRl8hMbuDqZIcyrSTe9niJJuYLldRn/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>REQ-AASPAP01-001_Documento-de-Requisitos.docx</t>
+          <t>PCP-AASPAP01-001_Documento-de-Design.docx</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1kV_N6w7TU5Cwe5SYWL3tcptlcr4oazYt/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1MkxkyhMa5O4d9ee1JVYHNZV59BxiHU3m/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3253,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>REV-AASPAP01-001_Registro-de-Revisao-por-Pares.docx</t>
+          <t>PLA-AASPAP01-001_Plano-de-Projeto.docx</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1b2XcTr_rrP1ntnEzllbB2gHNdFaEaLsQ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1D7tchEQKaqeZMZ2vNNa0wgnXevI-Br8H/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TAP-AASPAP01-001_Termo-de-Abertura.docx</t>
+          <t>RAC-AASPAP01-001_Relatorio-de-Acompanhamento.docx</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1vj9arb9bNdy4z2DLV7U8sEbBp4GuIMHw/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/155bBfagbpaZdKxRSqXQzkmZSQkmCHNt0/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>VV-AASPAP01-001_Plano-de-VV.docx</t>
+          <t>RASTR-AASPAP01-001_Matriz-de-Rastreabilidade.docx</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3307,139 +3307,139 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11Vx-bMcQfovROo3RwVY7-dQClEVcFp1e/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1nqVdGrDD5CJ_3zPB3IehiBEhuDKSxZlS/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
+          <t>04_registros/AASP_Andamento-Processuais</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>andamentos_ApisParceiras.jpg</t>
+          <t>REL-VV-AASPAP01-001_Relatorio-de-Execucao-de-Testes.docx</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1di53G9P1RLs2VtusPoTRJay3fOG7c1L2/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1TzIWFlAfEpqwWO0JIF3DACKPzPgC2sPV/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
+          <t>04_registros/AASP_Andamento-Processuais</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>andamentos_arquitetura.svg</t>
+          <t>REQ-AASPAP01-001_Documento-de-Requisitos.docx</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>svg</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1hwULBFas2YSOqC3BIi0dVbGelx-U-Mp0/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1kV_N6w7TU5Cwe5SYWL3tcptlcr4oazYt/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
+          <t>04_registros/AASP_Andamento-Processuais</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>andamentos_historicoPreservado.jpeg</t>
+          <t>REV-AASPAP01-001_Registro-de-Revisao-por-Pares.docx</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>jpeg</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Nx8OtLH1th3lVs3pRHd1yJjZ-l5jsR4s/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1b2XcTr_rrP1ntnEzllbB2gHNdFaEaLsQ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
+          <t>04_registros/AASP_Andamento-Processuais</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>andamentos_historicoPreservado1.jpg</t>
+          <t>REV-AASPAP01-002_Registro-de-Revisao-por-Pares-por-Entrega.docx</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1zXIyrAtYHinI0oETDvC-PQ0sgF4Z6Fjy/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ijB8cHIMAWWH29ZHGjN2ByonolS_z-XE/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
+          <t>04_registros/AASP_Andamento-Processuais</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>andamentos_historicoPreservado2.jpg</t>
+          <t>TAP-AASPAP01-001_Termo-de-Abertura.docx</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1l8sW0voE8k-y6ew1dTbd5aePqlr5UffM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1vj9arb9bNdy4z2DLV7U8sEbBp4GuIMHw/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
+          <t>04_registros/AASP_Andamento-Processuais</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>andamentos_retry_webhook.jpeg</t>
+          <t>VV-AASPAP01-001_Plano-de-VV.docx</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>jpeg</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15lXDLmdWW620DS2qE9-qwIEzvAgmpGlW/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/11Vx-bMcQfovROo3RwVY7-dQClEVcFp1e/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3451,17 +3451,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>devops_andamentos_branches.png</t>
+          <t>andamentos_ApisParceiras.jpg</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1YaLDEwp8l6FoyFTaMTEWMmeLqbT6gfnx/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1di53G9P1RLs2VtusPoTRJay3fOG7c1L2/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3473,17 +3473,17 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>devops_andamentos_commits.png</t>
+          <t>andamentos_arquitetura.svg</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>svg</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1fkX4bzm8iFGVFOtMtIK4rEtjZhF1bomY/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1hwULBFas2YSOqC3BIi0dVbGelx-U-Mp0/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3495,17 +3495,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>devops_andamentos_estrutura.png</t>
+          <t>andamentos_historicoPreservado.jpeg</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpeg</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1w_Hj4o0YyA0oYRSE1_5d1VE67_JisEFY/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Nx8OtLH1th3lVs3pRHd1yJjZ-l5jsR4s/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3517,17 +3517,17 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>devops_andamentos_pipeline_ci.png</t>
+          <t>andamentos_historicoPreservado1.jpg</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1p1VezDp1C0XYPSOjQk978cQmrvGVrTWo/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1zXIyrAtYHinI0oETDvC-PQ0sgF4Z6Fjy/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3539,17 +3539,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>devops_andamentos_pipeline_cicd.png</t>
+          <t>andamentos_historicoPreservado2.jpg</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Zf1k0e36NnyOxq-zv6Rrz22N5tvM8x49/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1l8sW0voE8k-y6ew1dTbd5aePqlr5UffM/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3561,17 +3561,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>devops_andamentos_pr_detail_1.png</t>
+          <t>andamentos_retry_webhook.jpeg</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpeg</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FSv2kmZbKNXOk5tjctohUFqHtn-BZ9bu/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/15lXDLmdWW620DS2qE9-qwIEzvAgmpGlW/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>devops_andamentos_pr_detail_2.png</t>
+          <t>devops_andamentos_branches.png</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1oBhgj_wDBy_Ap5QoTy-HRRu7a62wsa6S/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1YaLDEwp8l6FoyFTaMTEWMmeLqbT6gfnx/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>devops_andamentos_prs.png</t>
+          <t>devops_andamentos_commits.png</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/14Se4mDLpHgV5EjT8w7kd1TypMmOEmzMU/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1fkX4bzm8iFGVFOtMtIK4rEtjZhF1bomY/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>devops_andamentos_tags.png</t>
+          <t>devops_andamentos_estrutura.png</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1fGjCYwKyDczuhAJPkpaxCMdrrCi7BRc4/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1w_Hj4o0YyA0oYRSE1_5d1VE67_JisEFY/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>estrutura_andamentosProcessuais.png</t>
+          <t>devops_andamentos_pipeline_ci.png</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3659,139 +3659,139 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1BQ_7ZiscsMUDn84a_vBXcghhchm29hLs/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1p1VezDp1C0XYPSOjQk978cQmrvGVrTWo/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>04_registros/AASP_CNJ</t>
+          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>00_INDICEAASPCNJ01_MapadeRegistros.docx</t>
+          <t>devops_andamentos_pipeline_cicd.png</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1kf3EdS_AsVImdD6P_03zCt-OF7_UHj6N/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Zf1k0e36NnyOxq-zv6Rrz22N5tvM8x49/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>04_registros/AASP_CNJ</t>
+          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>ADAP-AASPCNJ01-001_Registro-de-Adaptacao.docx</t>
+          <t>devops_andamentos_pr_detail_1.png</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/14GFOTJj6jxDsV62h60zCqIgxnRW-DbWW/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1FSv2kmZbKNXOk5tjctohUFqHtn-BZ9bu/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>04_registros/AASP_CNJ</t>
+          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>ATA-AASPCNJ01-001_Ata-Alinhamento-Fluxo-CNJ.docx</t>
+          <t>devops_andamentos_pr_detail_2.png</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/12sOcC6FDaP-3OdoM1_duAMNNcbgYsQvb/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1oBhgj_wDBy_Ap5QoTy-HRRu7a62wsa6S/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>04_registros/AASP_CNJ</t>
+          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>CAP-AASPCNJ01-001_Registro-de-Capacitacao-da-Equipe.docx</t>
+          <t>devops_andamentos_prs.png</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11db2exVuX-huVhgL8azaDzByfMFQv_pb/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/14Se4mDLpHgV5EjT8w7kd1TypMmOEmzMU/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>04_registros/AASP_CNJ</t>
+          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>CR-AASPCNJ01-001_Change-Request.docx</t>
+          <t>devops_andamentos_tags.png</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1J3XOn56R7ruWa8vhPAnVzI7r092DFLY-/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1fGjCYwKyDczuhAJPkpaxCMdrrCi7BRc4/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>04_registros/AASP_CNJ</t>
+          <t>04_registros/AASP_Andamento-Processuais/evidencias</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>GCO-AASPCNJ01-001_Registro-de-Configuracao.docx</t>
+          <t>estrutura_andamentosProcessuais.png</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1IJozbK4BobNpyION4zPWa_s2auynxhv9/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1BQ_7ZiscsMUDn84a_vBXcghhchm29hLs/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>GDE-AASPCNJ01-001_Registro-de-Analise-de-Decisao.docx</t>
+          <t>00_INDICEAASPCNJ01_MapadeRegistros.docx</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1EpobYWmsjCftVdxosshioK0mCuXVFlEq/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1kf3EdS_AsVImdD6P_03zCt-OF7_UHj6N/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3825,17 +3825,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>GEST-AASPCNJ01-001_Planilha-de-Gestao-do-Projeto.xlsx</t>
+          <t>ADAP-AASPCNJ01-001_Registro-de-Adaptacao.docx</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Vdng-5mBCjlXpajdZ6ScLD67c8e85qob/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/14GFOTJj6jxDsV62h60zCqIgxnRW-DbWW/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>GQA-AASPCNJ01-001_Registro-de-GQA.docx</t>
+          <t>ATA-AASPCNJ01-001_Ata-Alinhamento-Fluxo-CNJ.docx</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1AI6TXKQ5f6Oh5g6VmFgzTmXNQHEtLOlh/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/12sOcC6FDaP-3OdoM1_duAMNNcbgYsQvb/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>ITP-AASPCNJ01-001_Estrategia-de-Integracao.docx</t>
+          <t>CAP-AASPCNJ01-001_Registro-de-Capacitacao-da-Equipe.docx</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1tobpnNoEQf5LarNnPEJAEJnt5BAZGrtQ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/11db2exVuX-huVhgL8azaDzByfMFQv_pb/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>MED-AASPCNJ01-001_Registro-de-Medicao.docx</t>
+          <t>CR-AASPCNJ01-001_Change-Request.docx</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ePiJ3ONIXZf2gN00FzXuyUCIXdrpezsx/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1J3XOn56R7ruWa8vhPAnVzI7r092DFLY-/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>PCP-AASPCNJ01-001_Documento-de-Design.docx</t>
+          <t>GCO-AASPCNJ01-001_Registro-de-Configuracao.docx</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ywDtDrM3zHptY2XfL6ut22ra3MEbuLTe/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1IJozbK4BobNpyION4zPWa_s2auynxhv9/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PLA-AASPCNJ01-001_Plano-de-Projeto.docx</t>
+          <t>GDE-AASPCNJ01-001_Registro-de-Analise-de-Decisao.docx</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1y9zo8Fx1AewE2z9GVdmhsecKySyDoSf6/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1EpobYWmsjCftVdxosshioK0mCuXVFlEq/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3957,17 +3957,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>RAC-AASPCNJ01-001_Relatorio-de-Acompanhamento.docx</t>
+          <t>GEST-AASPCNJ01-001_Planilha-de-Gestao-do-Projeto.xlsx</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1G_0Odyq4HbI3nfCyDh7-zZoXDgu_BiON/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Vdng-5mBCjlXpajdZ6ScLD67c8e85qob/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>RASTR-AASPCNJ01-001_Matriz-de-Rastreabilidade.docx</t>
+          <t>GQA-AASPCNJ01-001_Registro-de-GQA.docx</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3989,7 +3989,7 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1lfPyboZZ3hd-8g3IzjQRQciVYXCztgZw/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1AI6TXKQ5f6Oh5g6VmFgzTmXNQHEtLOlh/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>REL-VV-AASPCNJ01-001_Relatorio-de-Execucao-de-Testes.docx</t>
+          <t>ITP-AASPCNJ01-001_Estrategia-de-Integracao.docx</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1whC8gTS2Mz1CW7QajDlOMvfXNlxt5AP6/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1tobpnNoEQf5LarNnPEJAEJnt5BAZGrtQ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>REQ-AASPCNJ01-001_Documento-de-Requisitos.docx</t>
+          <t>MED-AASPCNJ01-001_Registro-de-Medicao.docx</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1GDwHhtK1Nc-2AptWo8HIryVHeOF8hzj5/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ePiJ3ONIXZf2gN00FzXuyUCIXdrpezsx/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4045,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>REV-AASPCNJ01-001_Registro-de-Revisao-por-Pares.docx</t>
+          <t>PCP-AASPCNJ01-001_Documento-de-Design.docx</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1PfM9kKAjFJofhtJn5xqgicqG-0-v3mA-/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ywDtDrM3zHptY2XfL6ut22ra3MEbuLTe/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>TAP-AASPCNJ01-001_Termo-de-Abertura.docx</t>
+          <t>PLA-AASPCNJ01-001_Plano-de-Projeto.docx</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1hKBUW2dTTfmd8PEs36tEuIQjsKjPAuRF/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1y9zo8Fx1AewE2z9GVdmhsecKySyDoSf6/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4089,7 +4089,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>VV-AASPCNJ01-001_Plano-de-VV.docx</t>
+          <t>RAC-AASPCNJ01-001_Relatorio-de-Acompanhamento.docx</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4099,19 +4099,19 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/199h316ZoZ43k7W_rnPpNq6GTBr502zuu/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1G_0Odyq4HbI3nfCyDh7-zZoXDgu_BiON/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/AASP_CNJ</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>ADAP-FRUKI01-001_Registro-de-Adaptacao.docx</t>
+          <t>RASTR-AASPCNJ01-001_Matriz-de-Rastreabilidade.docx</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4121,19 +4121,19 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1NaEJlUDHw0FE6fgH28gpifHft7ZLxUyL/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1lfPyboZZ3hd-8g3IzjQRQciVYXCztgZw/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/AASP_CNJ</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>ADAP-FRUKI01-002_Registro-de-Adaptacao-PacoteFinal24.docx</t>
+          <t>REL-VV-AASPCNJ01-001_Relatorio-de-Execucao-de-Testes.docx</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4143,19 +4143,19 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LNzyoQkTM7oLgWtSCPY6VxNqt4JS_MzM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1whC8gTS2Mz1CW7QajDlOMvfXNlxt5AP6/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/AASP_CNJ</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-001_Ata-de-Kickoff.docx</t>
+          <t>REQ-AASPCNJ01-001_Documento-de-Requisitos.docx</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4165,19 +4165,19 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pjAXblbrxR8Y6p5eq2BDYRBpiYlK3Ag_/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1GDwHhtK1Nc-2AptWo8HIryVHeOF8hzj5/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/AASP_CNJ</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-002_Ata-Levantamento-Metas.docx</t>
+          <t>REV-AASPCNJ01-001_Registro-de-Revisao-por-Pares.docx</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4187,19 +4187,19 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1cypxWHL-NU9CPnLV47N-bKnP0QrSIB17/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1PfM9kKAjFJofhtJn5xqgicqG-0-v3mA-/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/AASP_CNJ</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-003_Ata-de-Aceite-Final.docx</t>
+          <t>TAP-AASPCNJ01-001_Termo-de-Abertura.docx</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -4209,19 +4209,19 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1m0odZUeHy212r9AQwyZ_sfwXzznT4oqJ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1hKBUW2dTTfmd8PEs36tEuIQjsKjPAuRF/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/AASP_CNJ</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-004_Ata-Validacao-Sprint1-NaoAlocados.docx</t>
+          <t>VV-AASPCNJ01-001_Plano-de-VV.docx</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10Qo6yB8nqAQmzacMbuLZaVv1ZaX178Lt/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/199h316ZoZ43k7W_rnPpNq6GTBr502zuu/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-005_Ata-Validacao-Sprint2-RegraDeOuro.docx</t>
+          <t>ADAP-FRUKI01-001_Registro-de-Adaptacao.docx</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1VmGwsZK4GLu_zpzmrHnD2XOChsiR1GZr/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1NaEJlUDHw0FE6fgH28gpifHft7ZLxUyL/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-006_Ata-Validacao-Sprint3-PDV.docx</t>
+          <t>ADAP-FRUKI01-002_Registro-de-Adaptacao-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ujgsYTHnAVE_J60APn-OqGSRaCTbfPHf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1LNzyoQkTM7oLgWtSCPY6VxNqt4JS_MzM/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-007_Ata-Piloto-Pacote1.docx</t>
+          <t>ATA-FRUKI01-001_Ata-de-Kickoff.docx</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1bNAl7ljD0PhTyZEb-2ngdIbBzCpvNY2q/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1pjAXblbrxR8Y6p5eq2BDYRBpiYlK3Ag_/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>ATAFRUKI01008_AtaKickoffPacoteFinal24.docx</t>
+          <t>ATA-FRUKI01-002_Ata-Levantamento-Metas.docx</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11alVpwlnsPjgd1_PO4OzMBXeJLRz6PXi/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1cypxWHL-NU9CPnLV47N-bKnP0QrSIB17/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4331,17 +4331,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>AnaliseDecisao_FTFRUKI_TIMEWARE.xlsx</t>
+          <t>ATA-FRUKI01-003_Ata-de-Aceite-Final.docx</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19sYcZ40SHiEe7qUV7jau-3fruYrAzjWp/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1m0odZUeHy212r9AQwyZ_sfwXzznT4oqJ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CR-FRUKI01-001_Solicitacao-de-Mudanca-RegraDeOuro.docx</t>
+          <t>ATA-FRUKI01-004_Ata-Validacao-Sprint1-NaoAlocados.docx</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1z2TIuyQQTiU7fOKmK0kQfziTtE8NqiLc/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/10Qo6yB8nqAQmzacMbuLZaVv1ZaX178Lt/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>GCO-FRUKI01-001_Registro-de-Configuracao.docx</t>
+          <t>ATA-FRUKI01-005_Ata-Validacao-Sprint2-RegraDeOuro.docx</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1fMcui7ebx_4af41JtRltlCCJzDWkd1eA/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1VmGwsZK4GLu_zpzmrHnD2XOChsiR1GZr/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>GDE-FRUKI01-001_Registro-de-Decisao.docx</t>
+          <t>ATA-FRUKI01-006_Ata-Validacao-Sprint3-PDV.docx</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1h8FKsNP59PnO8tzm2WEJ_vgsZYRSmjwX/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ujgsYTHnAVE_J60APn-OqGSRaCTbfPHf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4419,17 +4419,17 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>GEST-FRUKI01-001_Planilha-de-Gestao-do-Projeto.xlsx</t>
+          <t>ATA-FRUKI01-007_Ata-Piloto-Pacote1.docx</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1RsktvVNbrH1f-RmcV3_AmIu3uJt9Q7sH/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1bNAl7ljD0PhTyZEb-2ngdIbBzCpvNY2q/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>GQA-FRUKI01-001_Registro-de-GQA.docx</t>
+          <t>ATAFRUKI01008_AtaKickoffPacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1jmdev8ggRDsbM_CrkMQY_oKaImvKG4vM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/11alVpwlnsPjgd1_PO4OzMBXeJLRz6PXi/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4463,17 +4463,17 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>ITP-FRUKI01-001_Estrategia-de-Integracao.docx</t>
+          <t>AnaliseDecisao_FTFRUKI_TIMEWARE.xlsx</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19YCw05XWIRh-NaI5GWf1c-MF6m5AhIra/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/19sYcZ40SHiEe7qUV7jau-3fruYrAzjWp/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>ITP-FRUKI01-002_Estrategia-de-Integracao-PacoteFinal24.docx</t>
+          <t>CR-FRUKI01-001_Solicitacao-de-Mudanca-RegraDeOuro.docx</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1A-6S0ZZmHteTzIjSNP46H2OJYgeI-Gc7/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1z2TIuyQQTiU7fOKmK0kQfziTtE8NqiLc/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>LI-FRUKI01-001_Licoes-Aprendidas.docx</t>
+          <t>GCO-FRUKI01-001_Registro-de-Configuracao.docx</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pXvWCErdbUdvvAcXV93935DeGW6bJ7xL/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1fMcui7ebx_4af41JtRltlCCJzDWkd1eA/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>MED-FRUKI01-001_Registro-de-Medicao.docx</t>
+          <t>GDE-FRUKI01-001_Registro-de-Decisao.docx</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1D6gCK_SBP31WdmYGToQH2iCZV1RdzhWI/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1h8FKsNP59PnO8tzm2WEJ_vgsZYRSmjwX/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4551,17 +4551,17 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>PCP-FRUKI01-001_Documento-de-Design.docx</t>
+          <t>GEST-FRUKI01-001_Planilha-de-Gestao-do-Projeto.xlsx</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ff6Ha1FH1T1XAJGnmdy2QvkrqXxCUg2s/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1RsktvVNbrH1f-RmcV3_AmIu3uJt9Q7sH/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>PCP-FRUKI01-002_Documento-de-Design-PacoteFinal24.docx</t>
+          <t>GQA-FRUKI01-001_Registro-de-GQA.docx</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17KodAvypysQkbqocfQIrlE2q1dfRIUnY/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1jmdev8ggRDsbM_CrkMQY_oKaImvKG4vM/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>PLA-FRUKI01-001_Plano-de-Projeto.docx</t>
+          <t>ITP-FRUKI01-001_Estrategia-de-Integracao.docx</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1WEPaZNg7rxj29B48l_scz7x7CyLlvoSf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/19YCw05XWIRh-NaI5GWf1c-MF6m5AhIra/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>PLA-FRUKI01-002_Plano-de-Projeto-PacoteFinal24.docx</t>
+          <t>ITP-FRUKI01-002_Estrategia-de-Integracao-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1d0l6IhtfbI9hE0UYxQm6nVq9grpjKnpn/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1A-6S0ZZmHteTzIjSNP46H2OJYgeI-Gc7/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>RAC-FRUKI01-001_Relatorio-de-Acompanhamento.docx</t>
+          <t>LI-FRUKI01-001_Licoes-Aprendidas.docx</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1_C3hZUp-7-2ldAa2BmIfZ3tMfa9WX0bd/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1pXvWCErdbUdvvAcXV93935DeGW6bJ7xL/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>RASTR-FRUKI01-001_Matriz-de-Rastreabilidade.docx</t>
+          <t>MED-FRUKI01-001_Registro-de-Medicao.docx</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1SokajsndvgCtPAX7FyUpNp9mIDxQrVQf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1D6gCK_SBP31WdmYGToQH2iCZV1RdzhWI/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>RASTR-FRUKI01-002_Matriz-de-Rastreabilidade-PacoteFinal24.docx</t>
+          <t>PCP-FRUKI01-001_Documento-de-Design.docx</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1S4nR_PkZnGQrm6ppWv47ftgH2ptyG9xJ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ff6Ha1FH1T1XAJGnmdy2QvkrqXxCUg2s/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>REQ-FRUKI01-001_Documento-de-Requisitos.docx</t>
+          <t>PCP-FRUKI01-002_Documento-de-Design-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1mCQ9GroaEFEjulblg31P0Kdknw95w8LJ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17KodAvypysQkbqocfQIrlE2q1dfRIUnY/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>REQ-FRUKI01-002_Documento-de-Requisitos-PacoteFinal24.docx</t>
+          <t>PLA-FRUKI01-001_Plano-de-Projeto.docx</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1GexOXykQE4rnKFPmeW1kVQac18vsnlnQ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1WEPaZNg7rxj29B48l_scz7x7CyLlvoSf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>TAE-FRUKI01-001_Termo-de-Encerramento.docx</t>
+          <t>PLA-FRUKI01-002_Plano-de-Projeto-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JNvLtWIaqno7WXqzPfQwcK1bRE3UjCRv/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1d0l6IhtfbI9hE0UYxQm6nVq9grpjKnpn/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>TAE-FRUKI01-002_Termo-de-Encerramento-PacoteFinal24.docx</t>
+          <t>RAC-FRUKI01-001_Relatorio-de-Acompanhamento.docx</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1D3T0RHrOPhOq08Edxc1fWW-cZ1uR-e2n/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1_C3hZUp-7-2ldAa2BmIfZ3tMfa9WX0bd/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>TAP-FRUKI01-001_Termo-de-Abertura.docx</t>
+          <t>RASTR-FRUKI01-001_Matriz-de-Rastreabilidade.docx</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ehO_9gQoPrLS-Ykhxfnnsrn9KZ9o8zdH/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1SokajsndvgCtPAX7FyUpNp9mIDxQrVQf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>TAP-FRUKI01-002_Termo-de-Abertura-PacoteFinal24.docx</t>
+          <t>RASTR-FRUKI01-002_Matriz-de-Rastreabilidade-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UUmn_lYKBv8eG5UZBaLipFbSMdnYTxgU/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1S4nR_PkZnGQrm6ppWv47ftgH2ptyG9xJ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4837,7 +4837,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>VV-FRUKI01-001_Plano-VeV.docx</t>
+          <t>REQ-FRUKI01-001_Documento-de-Requisitos.docx</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yCFY98oM8rlf44HUIeERib4_7jtYsKeU/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1mCQ9GroaEFEjulblg31P0Kdknw95w8LJ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>VV-FRUKI01-002_Plano-VeV-PacoteFinal24.docx</t>
+          <t>REQ-FRUKI01-002_Documento-de-Requisitos-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -4869,19 +4869,19 @@
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1d_okleyBKoPtPW2zEy7300KiXoWL62oj/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1GexOXykQE4rnKFPmeW1kVQac18vsnlnQ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>ADAP-GASMIG02-001_Registro-de-Adaptacao.docx</t>
+          <t>TAE-FRUKI01-001_Termo-de-Encerramento.docx</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -4891,19 +4891,19 @@
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1uDnjyU3hDOdzbVZPUFA-1PGqXCsuDeS7/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1JNvLtWIaqno7WXqzPfQwcK1bRE3UjCRv/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>ADAP-GASMIG02-002_Registro-de-Adaptacao-OS002.docx</t>
+          <t>TAE-FRUKI01-002_Termo-de-Encerramento-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -4913,19 +4913,19 @@
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1oQshhvn5DIq1DoB3rybc8jEbP_OdEnfn/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1D3T0RHrOPhOq08Edxc1fWW-cZ1uR-e2n/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>ATA-GASMIG02-001_Ata-de-Kickoff.docx</t>
+          <t>TAP-FRUKI01-001_Termo-de-Abertura.docx</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -4935,19 +4935,19 @@
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1XcstqfQTQC0cm8wZgfc9oLgjSknU6Ueq/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ehO_9gQoPrLS-Ykhxfnnsrn9KZ9o8zdH/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>ATA-GASMIG02-002_Ata-de-Aceite-OS001.docx</t>
+          <t>TAP-FRUKI01-002_Termo-de-Abertura-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -4957,19 +4957,19 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1CcRbEbIcDWeHO7sOznH_FcuK-uVVusM0/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1UUmn_lYKBv8eG5UZBaLipFbSMdnYTxgU/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>ATA-GASMIG02-003_Apresentacao-Entrega-OS002.docx</t>
+          <t>VV-FRUKI01-001_Plano-VeV.docx</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -4979,29 +4979,29 @@
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1YCW3PFHS2p1bh8O6VWyZ8y2NFoG6ZWFN/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1yCFY98oM8rlf44HUIeERib4_7jtYsKeU/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>AnaliseDecisao_FTGASMIG_TIMEWARE.xlsx</t>
+          <t>VV-FRUKI01-002_Plano-VeV-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1u5oCqJrnQuaPBUMqTNQvaukwxqZvsmQi/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1d_okleyBKoPtPW2zEy7300KiXoWL62oj/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>CAP-GASMIG02-001_Registro-de-Capacitacao-da-Equipe.docx</t>
+          <t>ADAP-GASMIG02-001_Registro-de-Adaptacao.docx</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ibleg7tRQDHfYp3ahRpAlbYjKetFDzzT/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1uDnjyU3hDOdzbVZPUFA-1PGqXCsuDeS7/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>GCO-GASMIG02-001_Gerencia-de-Configuracao.docx</t>
+          <t>ADAP-GASMIG02-002_Registro-de-Adaptacao-OS002.docx</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1qpIzDVbsmVYkiXW9NNdciOuv5iovMNu4/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1oQshhvn5DIq1DoB3rybc8jEbP_OdEnfn/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5057,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>GDE-GASMIG02-001_Registro-de-Analise-de-Decisao.docx</t>
+          <t>ATA-GASMIG02-001_Ata-de-Kickoff.docx</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1sqAtX-R1-EjASMtMCnp_fjiessTaSaQU/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1XcstqfQTQC0cm8wZgfc9oLgjSknU6Ueq/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5079,17 +5079,17 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>GEST-GASMIG02_Planilha-de-Gestao-do-Projeto.xlsx</t>
+          <t>ATA-GASMIG02-002_Ata-de-Aceite-OS001.docx</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1r_dSFP9AmEnj79FkmqU80OkuYWnwzfZS/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1CcRbEbIcDWeHO7sOznH_FcuK-uVVusM0/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>GQA-GASMIG02-001_Registro-de-GQA.docx</t>
+          <t>ATA-GASMIG02-003_Apresentacao-Entrega-OS002.docx</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1V-T1g_9AKu9TLFPROMR0fA1gkyx180a-/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1YCW3PFHS2p1bh8O6VWyZ8y2NFoG6ZWFN/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5123,17 +5123,17 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>ITP-GASMIG02-002_Estrategia-de-Integracao-OS002.docx</t>
+          <t>AnaliseDecisao_FTGASMIG_TIMEWARE.xlsx</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JIAbQHVpTSO3V0AKGnWyVwEs6zuTWX7R/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1u5oCqJrnQuaPBUMqTNQvaukwxqZvsmQi/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>LI-GASMIG02-001_Licoes-Aprendidas.docx</t>
+          <t>CAP-GASMIG02-001_Registro-de-Capacitacao-da-Equipe.docx</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -5155,7 +5155,7 @@
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ra9yyJuVYa2tmQW0DKwbJgannxAI2W0E/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ibleg7tRQDHfYp3ahRpAlbYjKetFDzzT/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5167,7 +5167,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>MED-GASMIG02-001_Registro-de-Medicao.docx</t>
+          <t>GCO-GASMIG02-001_Gerencia-de-Configuracao.docx</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LtjN_WSjn_g1wQ_RRLe4Z4KP6Cnu-Ohx/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1qpIzDVbsmVYkiXW9NNdciOuv5iovMNu4/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>PCP-GASMIG02-001_Documento-de-Design.docx</t>
+          <t>GDE-GASMIG02-001_Registro-de-Analise-de-Decisao.docx</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1YI-40O6IWGMB0C_R6ytpbxc2w1E7W4fF/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1sqAtX-R1-EjASMtMCnp_fjiessTaSaQU/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5211,17 +5211,17 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>PCP-GASMIG02-002_Documento-de-Design-OS002.docx</t>
+          <t>GEST-GASMIG02_Planilha-de-Gestao-do-Projeto.xlsx</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Q4M2R4uqiy81BP8L3HiQ_idRqmpMt8Cw/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1r_dSFP9AmEnj79FkmqU80OkuYWnwzfZS/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>PLA-GASMIG02-001_Plano-de-Projeto.docx</t>
+          <t>GQA-GASMIG02-001_Registro-de-GQA.docx</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ZIwX-h0RDNJfhO5AXev2vqhYrGHOr2qf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1V-T1g_9AKu9TLFPROMR0fA1gkyx180a-/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>PLA-GASMIG02-002_Plano-de-Projeto-OS002.docx</t>
+          <t>ITP-GASMIG02-002_Estrategia-de-Integracao-OS002.docx</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1jfUDk7bhCtOXUYDcBnpjOx8FARp2VqPH/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1JIAbQHVpTSO3V0AKGnWyVwEs6zuTWX7R/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>RAC-GASMIG02-001_Relatorio-de-Acompanhamento.docx</t>
+          <t>LI-GASMIG02-001_Licoes-Aprendidas.docx</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1bAl8o8UPkTb1AHypGNvRxEJG8UYswpvS/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ra9yyJuVYa2tmQW0DKwbJgannxAI2W0E/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>RASTR-GASMIG02-001_Matriz-de-Rastreabilidade.docx</t>
+          <t>MED-GASMIG02-001_Registro-de-Medicao.docx</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5309,7 +5309,7 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1_delTbo-PEeRpuGGGagv5p2SOF-ZNRos/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1LtjN_WSjn_g1wQ_RRLe4Z4KP6Cnu-Ohx/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>RASTR-GASMIG02-002_Matriz-de-Rastreabilidade-OS002.docx</t>
+          <t>PCP-GASMIG02-001_Documento-de-Design.docx</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1tfy9oNEOsThCKNb1YrvQq8Ll1jX9kYJO/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1YI-40O6IWGMB0C_R6ytpbxc2w1E7W4fF/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>REQ-GASMIG02-001_Documento-de-Requisitos.docx</t>
+          <t>PCP-GASMIG02-002_Documento-de-Design-OS002.docx</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/13duq0igfGKvJAHKh_sD9TN7WqTpuOfdn/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Q4M2R4uqiy81BP8L3HiQ_idRqmpMt8Cw/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>REQ-GASMIG02-002_Documento-de-Requisitos-OS002.docx</t>
+          <t>PLA-GASMIG02-001_Plano-de-Projeto.docx</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1_yN7yHPBc9iKilAlxd4pxj52G1_WoCHP/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ZIwX-h0RDNJfhO5AXev2vqhYrGHOr2qf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5387,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>REV-GASMIG02-001_Registro-de-Verificacao-Tecnica.docx</t>
+          <t>PLA-GASMIG02-002_Plano-de-Projeto-OS002.docx</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1biHfNjSf_g7hnUcjBATCG48aG7ARNvRL/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1jfUDk7bhCtOXUYDcBnpjOx8FARp2VqPH/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>TAE-GASMIG02-001_Termo-de-Encerramento-OS001.docx</t>
+          <t>RAC-GASMIG02-001_Relatorio-de-Acompanhamento.docx</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1mw7eJBj6HANyIYJ1MgxEnO59ML9sl5aa/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1bAl8o8UPkTb1AHypGNvRxEJG8UYswpvS/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>TAE-GASMIG02-002_Termo-de-Encerramento-OS002.docx</t>
+          <t>RASTR-GASMIG02-001_Matriz-de-Rastreabilidade.docx</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1-zvT45vPsVTAwmcEzQVak8qKT4dnQWEr/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1_delTbo-PEeRpuGGGagv5p2SOF-ZNRos/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5453,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>TAP-GASMIG02-001_Termo-de-Abertura.docx</t>
+          <t>RASTR-GASMIG02-002_Matriz-de-Rastreabilidade-OS002.docx</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -5463,7 +5463,7 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1WW3VNRafS44JkZiXK29Rm7bYI7NbP9rS/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1tfy9oNEOsThCKNb1YrvQq8Ll1jX9kYJO/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>TAP-GASMIG02-002_Termo-de-Abertura-OS002.docx</t>
+          <t>REQ-GASMIG02-001_Documento-de-Requisitos.docx</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1cMUOhgzZzj6wwWIijFMDugRVZIl8aPvf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/13duq0igfGKvJAHKh_sD9TN7WqTpuOfdn/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>VV-GASMIG02-001_Plano-de-VV.docx</t>
+          <t>REQ-GASMIG02-002_Documento-de-Requisitos-OS002.docx</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15t1yh5oMbpFZ47rREDx9kJPgS8oXyRmy/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1_yN7yHPBc9iKilAlxd4pxj52G1_WoCHP/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5519,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>VV-GASMIG02-002_Plano-de-VV-OS002.docx</t>
+          <t>REV-GASMIG02-001_Registro-de-Verificacao-Tecnica.docx</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -5529,19 +5529,19 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/18GgauiJykVy8AASSKtJcqkt2FR-6AuRv/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1biHfNjSf_g7hnUcjBATCG48aG7ARNvRL/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>ADAP-PROFARMA01-001_Registro-de-Adaptacao.docx</t>
+          <t>TAE-GASMIG02-001_Termo-de-Encerramento-OS001.docx</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5551,19 +5551,19 @@
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aRgkciq4Ed3iPJgEbe1jJnpkXKlF4Tma/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1mw7eJBj6HANyIYJ1MgxEnO59ML9sl5aa/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>ATA-PROFARMA01-001_Ata-de-Kickoff.docx</t>
+          <t>TAE-GASMIG02-002_Termo-de-Encerramento-OS002.docx</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -5573,19 +5573,19 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1uNkVDge5WAgwLTCcUFZmBLlqKog16nmG/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1-zvT45vPsVTAwmcEzQVak8qKT4dnQWEr/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>ATA-PROFARMA01-002_Ata-de-Aceite-Final.docx</t>
+          <t>TAP-GASMIG02-001_Termo-de-Abertura.docx</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -5595,41 +5595,41 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1odIVE62I5L7iqqLFUCACbHt3w2HRB8yR/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1WW3VNRafS44JkZiXK29Rm7bYI7NbP9rS/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Analise-Decisao_PROFARMA_TIMEWARE.xlsx</t>
+          <t>TAP-GASMIG02-002_Termo-de-Abertura-OS002.docx</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1iS1LRiviBLZgmxymc7Hfq7szzjUGkHjK/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1cMUOhgzZzj6wwWIijFMDugRVZIl8aPvf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>CR-PROFARMA01-001_Registro-de-Change-Requests.docx</t>
+          <t>VV-GASMIG02-001_Plano-de-VV.docx</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -5639,19 +5639,19 @@
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1XWRRoeJ6NnvjCG3S0hlyPyxnMfkf9vM7/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/15t1yh5oMbpFZ47rREDx9kJPgS8oXyRmy/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+          <t>04_registros/FTGASMIG_Governanca-APIs/GASMIG02_Fundacao-Tecnologica</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>CTQ-PROFARMA01-001_Cenarios-de-Teste-Homologacao.docx</t>
+          <t>VV-GASMIG02-002_Plano-de-VV-OS002.docx</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ts70FWbIasG3sf9qDBSw8cXldJfRJ7bY/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/18GgauiJykVy8AASSKtJcqkt2FR-6AuRv/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>EV-AzureDevOps-PROFARMA01-001.docx</t>
+          <t>ADAP-PROFARMA01-001_Registro-de-Adaptacao.docx</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1K3LjcxoNE5lRsuUe0IIkCtwreoj3Bizv/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1aRgkciq4Ed3iPJgEbe1jJnpkXKlF4Tma/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>EV-Jira-PROFARMA01-001.docx</t>
+          <t>ATA-PROFARMA01-001_Ata-de-Kickoff.docx</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ftGwgagbTkMohz_ZpKcLT0Z1_cPq_4A9/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1uNkVDge5WAgwLTCcUFZmBLlqKog16nmG/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>EV-Swagger-PROFARMA01-001.docx</t>
+          <t>ATA-PROFARMA01-002_Ata-de-Aceite-Final.docx</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17hu5hEzQctuc6OaDun7ki1pn1f-fp7cL/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1odIVE62I5L7iqqLFUCACbHt3w2HRB8yR/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5739,17 +5739,17 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>GCO-PROFARMA01-001_Registro-de-Gerencia-de-Configuracao.docx</t>
+          <t>Analise-Decisao_PROFARMA_TIMEWARE.xlsx</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ld1PXP0yafu0eW7nUNXN0iRCm1P7cskc/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1iS1LRiviBLZgmxymc7Hfq7szzjUGkHjK/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>GDE-PROFARMA01-001_Registro-de-Analise-de-Decisao.docx</t>
+          <t>CR-PROFARMA01-001_Registro-de-Change-Requests.docx</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1wU_hxVhwrX-XUT1OQmEKxw80Mz0T5Rat/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1XWRRoeJ6NnvjCG3S0hlyPyxnMfkf9vM7/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5783,17 +5783,17 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>GEST-PROFARMA01_Planilha-de-Gestao-do-Projeto.xlsx</t>
+          <t>CTQ-PROFARMA01-001_Cenarios-de-Teste-Homologacao.docx</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/12SEFOVCAA1jVQRgM1c1RDR_CL3KaW32_/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ts70FWbIasG3sf9qDBSw8cXldJfRJ7bY/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5805,7 +5805,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>GQA-PROFARMA01-001_Registro-de-GQA.docx</t>
+          <t>EV-AzureDevOps-PROFARMA01-001.docx</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -5815,7 +5815,7 @@
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1hefq-kmdiYVOIvc0RoWHcSVQDBbL8Fq4/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1K3LjcxoNE5lRsuUe0IIkCtwreoj3Bizv/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5827,7 +5827,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>ITP-PROFARMA01-001_Estrategia-de-Integracao.docx</t>
+          <t>EV-Jira-PROFARMA01-001.docx</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1DKKcqAZK78dkV2UIRRSXHtELjnxdw4aj/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ftGwgagbTkMohz_ZpKcLT0Z1_cPq_4A9/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5849,7 +5849,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>LI-PROFARMA01-001_Licoes-Aprendidas.docx</t>
+          <t>EV-Swagger-PROFARMA01-001.docx</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1NMayhfr_e6Li-R0NEGoST5QATJgifMc7/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17hu5hEzQctuc6OaDun7ki1pn1f-fp7cL/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>MED-PROFARMA01-001_Registro-de-Medicao.docx</t>
+          <t>GCO-PROFARMA01-001_Registro-de-Gerencia-de-Configuracao.docx</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nmbiWfvYMAAa7Y5pO14VxaZgxEPQuKOn/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ld1PXP0yafu0eW7nUNXN0iRCm1P7cskc/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>PCP-PROFARMA01-001_Documento-de-Design.docx</t>
+          <t>GDE-PROFARMA01-001_Registro-de-Analise-de-Decisao.docx</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1t0fD748MR_EBRMHsgQzVGLKRnJ4Zq7__/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1wU_hxVhwrX-XUT1OQmEKxw80Mz0T5Rat/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5915,17 +5915,17 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>PLA-PROFARMA01-001_Plano-de-Projeto.docx</t>
+          <t>GEST-PROFARMA01_Planilha-de-Gestao-do-Projeto.xlsx</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/189Kp-xA8BJ3SsO9NhxDyDOUtX3dADifK/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/12SEFOVCAA1jVQRgM1c1RDR_CL3KaW32_/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>RAC-PROFARMA01-001_Relatorio-de-Acompanhamento.docx</t>
+          <t>GQA-PROFARMA01-001_Registro-de-GQA.docx</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HjCxyFwvC7Fxp4OXwxjqqL7OyYlSfI9x/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1hefq-kmdiYVOIvc0RoWHcSVQDBbL8Fq4/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>RASTR-PROFARMA01-001_Matriz-de-Rastreabilidade.docx</t>
+          <t>ITP-PROFARMA01-001_Estrategia-de-Integracao.docx</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ep0JvVMNhdLVRwWXVMIyfLxurd7ReAyI/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1DKKcqAZK78dkV2UIRRSXHtELjnxdw4aj/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>REL-VV-PROFARMA01-001_Relatorio-de-Execucao-de-Testes.docx</t>
+          <t>LI-PROFARMA01-001_Licoes-Aprendidas.docx</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1KF8zj0lufb0VPg6riJwGhibojJJIopHM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1NMayhfr_e6Li-R0NEGoST5QATJgifMc7/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -6003,7 +6003,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>REQ-PROFARMA01-001_Documento-de-Requisitos.docx</t>
+          <t>MED-PROFARMA01-001_Registro-de-Medicao.docx</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17OE2PW4XkEy3OnJlSb6rtsHHh9ouTFJE/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1nmbiWfvYMAAa7Y5pO14VxaZgxEPQuKOn/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>REV-PROFARMA01-001_Registro-de-Revisao-Tecnica.docx</t>
+          <t>PCP-PROFARMA01-001_Documento-de-Design.docx</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1dHd-EpgVX2Mg2Wo5Y_uxB8KFH4qphhxM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1t0fD748MR_EBRMHsgQzVGLKRnJ4Zq7__/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>TAE-PROFARMA01-001_Termo-de-Encerramento.docx</t>
+          <t>PLA-PROFARMA01-001_Plano-de-Projeto.docx</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1k_UZ_jWRVmpHA1Iiysa7vKvUwQ1T8QED/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/189Kp-xA8BJ3SsO9NhxDyDOUtX3dADifK/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6069,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>TAP-PROFARMA01-001_Termo-de-Abertura.docx</t>
+          <t>RAC-PROFARMA01-001_Relatorio-de-Acompanhamento.docx</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6079,7 +6079,7 @@
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/13BKbRnLmlBDMBkioH54vOpmicKqlei8W/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1HjCxyFwvC7Fxp4OXwxjqqL7OyYlSfI9x/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6091,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>VV-PROFARMA01-001_Plano-de-VV.docx</t>
+          <t>RASTR-PROFARMA01-001_Matriz-de-Rastreabilidade.docx</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -6101,19 +6101,19 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15tRkpsMad47tD4gPdlLKImY5ipIadjxw/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ep0JvVMNhdLVRwWXVMIyfLxurd7ReAyI/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>05_capacidade</t>
+          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>MAPA-CAP-001_Mapa-de-Capacidade-dos-Processos.docx</t>
+          <t>REL-VV-PROFARMA01-001_Relatorio-de-Execucao-de-Testes.docx</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6123,19 +6123,19 @@
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17csazhVOlhhgaMN-DCmoQEUiJsfrN1Il/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1KF8zj0lufb0VPg6riJwGhibojJJIopHM/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>05_capacidade</t>
+          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>MAPA-ORG-001_Matriz-de-Papeis-e-Responsabilidades.docx</t>
+          <t>REQ-PROFARMA01-001_Documento-de-Requisitos.docx</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6145,34 +6145,166 @@
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1j98CQbhiUr74uV7VenwJcEhnLmLupxhe/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17OE2PW4XkEy3OnJlSb6rtsHHh9ouTFJE/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
+          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>REV-PROFARMA01-001_Registro-de-Revisao-Tecnica.docx</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dHd-EpgVX2Mg2Wo5Y_uxB8KFH4qphhxM/view?usp=drivesdk</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>TAE-PROFARMA01-001_Termo-de-Encerramento.docx</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1k_UZ_jWRVmpHA1Iiysa7vKvUwQ1T8QED/view?usp=drivesdk</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>TAP-PROFARMA01-001_Termo-de-Abertura.docx</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/13BKbRnLmlBDMBkioH54vOpmicKqlei8W/view?usp=drivesdk</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>04_registros/PROFARMA_Cadastro-de-Clientes</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>VV-PROFARMA01-001_Plano-de-VV.docx</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/15tRkpsMad47tD4gPdlLKImY5ipIadjxw/view?usp=drivesdk</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
           <t>05_capacidade</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr">
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>MAPA-CAP-001_Mapa-de-Capacidade-dos-Processos.docx</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/17csazhVOlhhgaMN-DCmoQEUiJsfrN1Il/view?usp=drivesdk</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>05_capacidade</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>MAPA-ORG-001_Matriz-de-Papeis-e-Responsabilidades.docx</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1j98CQbhiUr74uV7VenwJcEhnLmLupxhe/view?usp=drivesdk</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>05_capacidade</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
         <is>
           <t>MAPA-ORG-001_Matriz-de-Papeis-e-Responsabilidades.xlsx</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr">
+      <c r="C267" t="inlineStr">
         <is>
           <t>xlsx</t>
         </is>
       </c>
-      <c r="D261" s="2" t="inlineStr">
+      <c r="D267" s="2" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1i87bnTiddeMILoHq3CBlyZ-WzPS5meEW/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D261"/>
+  <autoFilter ref="A1:D267"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -6434,6 +6566,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId258"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId259"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId266"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza FTFRUKI: reestruturada em subpastas 00_Comum/Fase1/Fase2
A pasta FTFRUKI foi reorganizada: os 35 arquivos antes soltos (mae. .docx)
sairam da raiz; agora ha 35 arquivos em 3 subpastas, predominantemente .md.
Substituidas as 35 linhas antigas (links mortos) pelas atuais via search_files.

- 00_Comum: 6 (5 .md + 1 .xlsx)
- Fase1: 13 (.md)
- Fase2: 16 (.md)

Total do mapa permanece 266; muda a composicao: docx 228->195, md 0->34,
xlsx 12->11. Sem ids/documentos duplicados.

https://claude.ai/code/session_01Le3EZ8QjyEACMRtgYDCzkN
</commit_message>
<xml_diff>
--- a/MAPA-DRIVE_Indice-de-Links.xlsx
+++ b/MAPA-DRIVE_Indice-de-Links.xlsx
@@ -4238,770 +4238,770 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/00_Comum</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ADAP-FRUKI01-001_Registro-de-Adaptacao.docx</t>
+          <t>GCO-FRUKI01-001_Registro-de-Configuracao.md</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1NaEJlUDHw0FE6fgH28gpifHft7ZLxUyL/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1yZ7iuUvSlwsgPoGBWgXxDjKNTofdWRAu/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/00_Comum</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>ADAP-FRUKI01-002_Registro-de-Adaptacao-PacoteFinal24.docx</t>
+          <t>GDE-FRUKI01-001_Registro-de-Decisao.md</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LNzyoQkTM7oLgWtSCPY6VxNqt4JS_MzM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1hcn4AishYVOXgTA-qq--wQXfa5rN2J7j/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/00_Comum</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-001_Ata-de-Kickoff.docx</t>
+          <t>GQA-FRUKI01-001_Registro-de-GQA.md</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pjAXblbrxR8Y6p5eq2BDYRBpiYlK3Ag_/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Xhrg8NS3j_pN1Bv_z1Qo3009f_xVYYJx/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/00_Comum</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-002_Ata-Levantamento-Metas.docx</t>
+          <t>LI-FRUKI01-001_Licoes-Aprendidas.md</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1cypxWHL-NU9CPnLV47N-bKnP0QrSIB17/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1A_N6OJ8TlDnicQrSrnNfBOqLFzHl93cF/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/00_Comum</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-003_Ata-de-Aceite-Final.docx</t>
+          <t>MED-FRUKI01-001_Registro-de-Medicao.md</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1m0odZUeHy212r9AQwyZ_sfwXzznT4oqJ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1oQr_iKEzIYoU1ETYOAfRLqKmzOYWrE6P/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/00_Comum</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-004_Ata-Validacao-Sprint1-NaoAlocados.docx</t>
+          <t>RAC-FRUKI01-002_Planilha-de-Gestao-do-Projeto.xlsx</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10Qo6yB8nqAQmzacMbuLZaVv1ZaX178Lt/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ZwQgdrMLk96Yo2EyAtPobbt2i_FyGhxe/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-005_Ata-Validacao-Sprint2-RegraDeOuro.docx</t>
+          <t>ADAP-FRUKI01-001_Registro-de-Adaptacao.md</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1VmGwsZK4GLu_zpzmrHnD2XOChsiR1GZr/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1g-INZLVI4w9mctAzk6OGTBdLW39j5J-O/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-006_Ata-Validacao-Sprint3-PDV.docx</t>
+          <t>ATA-FRUKI01-001_Ata-de-Kickoff.md</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ujgsYTHnAVE_J60APn-OqGSRaCTbfPHf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1SIsT8G2rPxBsPHS_a34NVOkfIczIAbEO/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-007_Ata-Piloto-Pacote1.docx</t>
+          <t>ATA-FRUKI01-002_Ata-Levantamento-Metas.md</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1bNAl7ljD0PhTyZEb-2ngdIbBzCpvNY2q/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1JCWhoRHCOa43L1rL1y9xhz2bzFiioUnK/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>ATAFRUKI01008_AtaKickoffPacoteFinal24.docx</t>
+          <t>ATA-FRUKI01-007_Ata-Piloto-Pacote1.md</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11alVpwlnsPjgd1_PO4OzMBXeJLRz6PXi/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1i2TY8dz01qak1BldOVjMBL1BjH02Lnuv/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>AnaliseDecisao_FTFRUKI_TIMEWARE.xlsx</t>
+          <t>ITP-FRUKI01-001_Estrategia-de-Integracao.md</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19sYcZ40SHiEe7qUV7jau-3fruYrAzjWp/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/11y80hz07nL5InEITjRl2F_pOMiDhlHKf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CR-FRUKI01-001_Solicitacao-de-Mudanca-RegraDeOuro.docx</t>
+          <t>PCP-FRUKI01-001_Documento-de-Design.md</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1z2TIuyQQTiU7fOKmK0kQfziTtE8NqiLc/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Lv68QFqybPvcG03VHmdEaL6dnBac8lSg/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>GCO-FRUKI01-001_Registro-de-Configuracao.docx</t>
+          <t>PLA-FRUKI01-001_Plano-de-Projeto.md</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1fMcui7ebx_4af41JtRltlCCJzDWkd1eA/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1nRlcB-Y-88Uwxc_7bC2AdBAF0kzWBaQv/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>GDE-FRUKI01-001_Registro-de-Decisao.docx</t>
+          <t>RAC-FRUKI01-002_Relatorio-de-Acompanhamento-Pacote1.md</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1h8FKsNP59PnO8tzm2WEJ_vgsZYRSmjwX/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1H6OwCNBXOpeXunhW1zRuov7QJ0ujUR2B/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>GEST-FRUKI01-001_Planilha-de-Gestao-do-Projeto.xlsx</t>
+          <t>RASTR-FRUKI01-001_Matriz-de-Rastreabilidade.md</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1RsktvVNbrH1f-RmcV3_AmIu3uJt9Q7sH/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1RlKVc6M0_sBlK9SoGVfJTxjGooTxQu5-/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>GQA-FRUKI01-001_Registro-de-GQA.docx</t>
+          <t>REQ-FRUKI01-001_Documento-de-Requisitos.md</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1jmdev8ggRDsbM_CrkMQY_oKaImvKG4vM/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1jsj6iEmqHQeFIV_2mbnVLU2yGk_aZSrG/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>ITP-FRUKI01-001_Estrategia-de-Integracao.docx</t>
+          <t>TAE-FRUKI01-001_Termo-de-Encerramento.md</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19YCw05XWIRh-NaI5GWf1c-MF6m5AhIra/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1eUVKAwQOSziboYim_LkDwdl-CRRKAkTE/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>ITP-FRUKI01-002_Estrategia-de-Integracao-PacoteFinal24.docx</t>
+          <t>TAP-FRUKI01-001_Termo-de-Abertura.md</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1A-6S0ZZmHteTzIjSNP46H2OJYgeI-Gc7/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1lyGciE7qckPltxEtVNXcwC2BbewYy8n8/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase1</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>LI-FRUKI01-001_Licoes-Aprendidas.docx</t>
+          <t>VV-FRUKI01-001_Plano-VeV.md</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pXvWCErdbUdvvAcXV93935DeGW6bJ7xL/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1pa1Kv-CVgiDKp6O15HsH2wS1Sj6w6rl2/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>MED-FRUKI01-001_Registro-de-Medicao.docx</t>
+          <t>ADAP-FRUKI01-002_Registro-de-Adaptacao-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1D6gCK_SBP31WdmYGToQH2iCZV1RdzhWI/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1gUQ1M-ZbVfLD2JDMMRy5dF-HwbZGqGT5/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>PCP-FRUKI01-001_Documento-de-Design.docx</t>
+          <t>ATA-FRUKI01-003_Ata-de-Aceite-Final.md</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ff6Ha1FH1T1XAJGnmdy2QvkrqXxCUg2s/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1-aeqT0BAQN8q9aiSFDprKncgUGv35Tbw/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>PCP-FRUKI01-002_Documento-de-Design-PacoteFinal24.docx</t>
+          <t>ATA-FRUKI01-004_Ata-Validacao-Sprint1-NaoAlocados.md</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17KodAvypysQkbqocfQIrlE2q1dfRIUnY/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/16-FiineTnD7qs-K0efjHI8oveh067Pjb/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>PLA-FRUKI01-001_Plano-de-Projeto.docx</t>
+          <t>ATA-FRUKI01-005_Ata-Validacao-Sprint2-RegraDeOuro.md</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1WEPaZNg7rxj29B48l_scz7x7CyLlvoSf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1pDeNymn8eEw1bg7neASDrMpjaHtKKF3m/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>PLA-FRUKI01-002_Plano-de-Projeto-PacoteFinal24.docx</t>
+          <t>ATA-FRUKI01-006_Ata-Validacao-Sprint3-PDV.md</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1d0l6IhtfbI9hE0UYxQm6nVq9grpjKnpn/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1tfZWSE26gCYWH3-cALxoyp66y9FEXp-R/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>RAC-FRUKI01-001_Relatorio-de-Acompanhamento.docx</t>
+          <t>ATA-FRUKI01-008_Ata-Kickoff-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1_C3hZUp-7-2ldAa2BmIfZ3tMfa9WX0bd/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1W-eIgotNpxwMJEQ3NO9CEQwVqcRKvOrq/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>RASTR-FRUKI01-001_Matriz-de-Rastreabilidade.docx</t>
+          <t>CR-FRUKI01-001_Solicitacao-de-Mudanca-RegraDeOuro.md</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1SokajsndvgCtPAX7FyUpNp9mIDxQrVQf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17fNk1TFIvfWh4C2O_pOGytMA5Gj9xgrr/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>RASTR-FRUKI01-002_Matriz-de-Rastreabilidade-PacoteFinal24.docx</t>
+          <t>ITP-FRUKI01-002_Estrategia-de-Integracao-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1S4nR_PkZnGQrm6ppWv47ftgH2ptyG9xJ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1b7z0ytGUrMuvUxixgK9g_YtzJOIAFlaD/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>REQ-FRUKI01-001_Documento-de-Requisitos.docx</t>
+          <t>PCP-FRUKI01-002_Documento-de-Design-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1mCQ9GroaEFEjulblg31P0Kdknw95w8LJ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17pKjVVEK0WOH8TP4tQrYY-1SEOD87_gn/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>REQ-FRUKI01-002_Documento-de-Requisitos-PacoteFinal24.docx</t>
+          <t>PLA-FRUKI01-002_Plano-de-Projeto-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1GexOXykQE4rnKFPmeW1kVQac18vsnlnQ/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/11HJg1b3_ko_YRr18_io0PeJKdqbBS6cz/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>TAE-FRUKI01-001_Termo-de-Encerramento.docx</t>
+          <t>RAC-FRUKI01-001_Relatorio-de-Acompanhamento.md</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JNvLtWIaqno7WXqzPfQwcK1bRE3UjCRv/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1tJKc9cSokMjVl6ZUEGziBPortQ0w9vHs/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>TAE-FRUKI01-002_Termo-de-Encerramento-PacoteFinal24.docx</t>
+          <t>RASTR-FRUKI01-002_Matriz-de-Rastreabilidade-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1D3T0RHrOPhOq08Edxc1fWW-cZ1uR-e2n/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1r2v_XLLzm37ySMynrN3AyLOGj1IHdnoW/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>TAP-FRUKI01-001_Termo-de-Abertura.docx</t>
+          <t>REQ-FRUKI01-002_Documento-de-Requisitos-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ehO_9gQoPrLS-Ykhxfnnsrn9KZ9o8zdH/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Fb7MpfzPfNKM--4N94Tx49pUGvWBnKab/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>TAP-FRUKI01-002_Termo-de-Abertura-PacoteFinal24.docx</t>
+          <t>TAE-FRUKI01-002_Termo-de-Encerramento-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UUmn_lYKBv8eG5UZBaLipFbSMdnYTxgU/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1qGo80blY7kzlFuXtUUCrkV6K427xB6SK/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>VV-FRUKI01-001_Plano-VeV.docx</t>
+          <t>TAP-FRUKI01-002_Termo-de-Abertura-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yCFY98oM8rlf44HUIeERib4_7jtYsKeU/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ngjegtxERo_jJObFfcYsUfNPw9yuC9PV/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas</t>
+          <t>04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/Fase2</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>VV-FRUKI01-002_Plano-VeV-PacoteFinal24.docx</t>
+          <t>VV-FRUKI01-002_Plano-VeV-PacoteFinal24.md</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1d_okleyBKoPtPW2zEy7300KiXoWL62oj/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1WcBf_hl4Unrs6FsG4AHhcJ-NuAoEG1s5/view?usp=drivesdk</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige FTFRUKI: refeita em .docx (subpastas recriadas, novos IDs)
FTFRUKI foi refeita: os .md anteriores foram substituidos por .docx, em
subpastas 00_Comum/Fase1/Fase2 recriadas (IDs novos). Re-mapeada via
search_files e substituidas as linhas .md (links mortos) pelas .docx atuais.

- 00_Comum: 6 (5 .docx + 1 .xlsx)
- Fase1: 13 (.docx)
- Fase2: 16 (.docx)

Total do mapa 266; composicao volta a docx 229, md 0, xlsx 11.
Sem ids/documentos duplicados.

https://claude.ai/code/session_01Le3EZ8QjyEACMRtgYDCzkN
</commit_message>
<xml_diff>
--- a/MAPA-DRIVE_Indice-de-Links.xlsx
+++ b/MAPA-DRIVE_Indice-de-Links.xlsx
@@ -4243,17 +4243,17 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>GCO-FRUKI01-001_Registro-de-Configuracao.md</t>
+          <t>GCO-FRUKI01-001_Registro-de-Configuracao.docx</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yZ7iuUvSlwsgPoGBWgXxDjKNTofdWRAu/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1pNtMiuOiFIaHQPJgi6eVfUg5n09WLqBP/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4265,17 +4265,17 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>GDE-FRUKI01-001_Registro-de-Decisao.md</t>
+          <t>GDE-FRUKI01-001_Registro-de-Decisao.docx</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1hcn4AishYVOXgTA-qq--wQXfa5rN2J7j/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1zmsr5YyHjrNpwEp90By_W7S1GnElYmw8/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4287,17 +4287,17 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>GQA-FRUKI01-001_Registro-de-GQA.md</t>
+          <t>GQA-FRUKI01-001_Registro-de-GQA.docx</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Xhrg8NS3j_pN1Bv_z1Qo3009f_xVYYJx/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1hmfL9793lOZ1GYNpydSIg3qi8_6Mw_Rg/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4309,17 +4309,17 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>LI-FRUKI01-001_Licoes-Aprendidas.md</t>
+          <t>LI-FRUKI01-001_Licoes-Aprendidas.docx</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1A_N6OJ8TlDnicQrSrnNfBOqLFzHl93cF/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17Qt_1yhKepTzL_g9JFOPU5J1Q2UF-BCX/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4331,17 +4331,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>MED-FRUKI01-001_Registro-de-Medicao.md</t>
+          <t>MED-FRUKI01-001_Registro-de-Medicao.docx</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1oQr_iKEzIYoU1ETYOAfRLqKmzOYWrE6P/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/14EdqCHT1X2JpRNN_NZ3C8Ews0ON8xu1P/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ZwQgdrMLk96Yo2EyAtPobbt2i_FyGhxe/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17ieOzpbIyysqF4xnATVsvILE3L3juD4Z/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4375,17 +4375,17 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>ADAP-FRUKI01-001_Registro-de-Adaptacao.md</t>
+          <t>ADAP-FRUKI01-001_Registro-de-Adaptacao.docx</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1g-INZLVI4w9mctAzk6OGTBdLW39j5J-O/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1efYcrr-1Tiw6JyKjakckma78t0SmY43G/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4397,17 +4397,17 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-001_Ata-de-Kickoff.md</t>
+          <t>ATA-FRUKI01-001_Ata-de-Kickoff.docx</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1SIsT8G2rPxBsPHS_a34NVOkfIczIAbEO/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1Ry0TUfXQPFqDBUkeeUNOk5vb3pDwIlVS/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4419,17 +4419,17 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-002_Ata-Levantamento-Metas.md</t>
+          <t>ATA-FRUKI01-002_Ata-Levantamento-Metas.docx</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JCWhoRHCOa43L1rL1y9xhz2bzFiioUnK/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1PnWtrFi4hLIWraOqhBVWpbOkJXFUMI9O/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4441,17 +4441,17 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-007_Ata-Piloto-Pacote1.md</t>
+          <t>ATA-FRUKI01-007_Ata-Piloto-Pacote1.docx</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1i2TY8dz01qak1BldOVjMBL1BjH02Lnuv/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/19h2hAuaXqPLMEIRQXXPIepH4F7aGuJqz/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4463,17 +4463,17 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>ITP-FRUKI01-001_Estrategia-de-Integracao.md</t>
+          <t>ITP-FRUKI01-001_Estrategia-de-Integracao.docx</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11y80hz07nL5InEITjRl2F_pOMiDhlHKf/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1vPddrPn96WUUiXuR-EYuaZqNwsD8kg4H/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4485,17 +4485,17 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>PCP-FRUKI01-001_Documento-de-Design.md</t>
+          <t>PCP-FRUKI01-001_Documento-de-Design.docx</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Lv68QFqybPvcG03VHmdEaL6dnBac8lSg/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1DhU-ouU4se-N_zNSd5WL1VHcuWwv7abA/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4507,17 +4507,17 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>PLA-FRUKI01-001_Plano-de-Projeto.md</t>
+          <t>PLA-FRUKI01-001_Plano-de-Projeto.docx</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nRlcB-Y-88Uwxc_7bC2AdBAF0kzWBaQv/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/18AHtQjHJ04e1unAbEuXyuSufSVAxy9np/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4529,17 +4529,17 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>RAC-FRUKI01-002_Relatorio-de-Acompanhamento-Pacote1.md</t>
+          <t>RAC-FRUKI01-002_Relatorio-de-Acompanhamento-Pacote1.docx</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1H6OwCNBXOpeXunhW1zRuov7QJ0ujUR2B/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1387oUWKKn_H3kKKKjDprHWcfJcHeunJy/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4551,17 +4551,17 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>RASTR-FRUKI01-001_Matriz-de-Rastreabilidade.md</t>
+          <t>RASTR-FRUKI01-001_Matriz-de-Rastreabilidade.docx</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1RlKVc6M0_sBlK9SoGVfJTxjGooTxQu5-/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/10vzbMMnDEc6da_gk6WMvbc_SoIkjaVPr/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4573,17 +4573,17 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>REQ-FRUKI01-001_Documento-de-Requisitos.md</t>
+          <t>REQ-FRUKI01-001_Documento-de-Requisitos.docx</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1jsj6iEmqHQeFIV_2mbnVLU2yGk_aZSrG/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/17zmKJI3e67wnxKzzzhVPhCZ3IxXBIFWU/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4595,17 +4595,17 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>TAE-FRUKI01-001_Termo-de-Encerramento.md</t>
+          <t>TAE-FRUKI01-001_Termo-de-Encerramento.docx</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1eUVKAwQOSziboYim_LkDwdl-CRRKAkTE/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1eI5-xDVUYZm1JfdD7jFDTmfgShwVcK16/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4617,17 +4617,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>TAP-FRUKI01-001_Termo-de-Abertura.md</t>
+          <t>TAP-FRUKI01-001_Termo-de-Abertura.docx</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1lyGciE7qckPltxEtVNXcwC2BbewYy8n8/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1hroxBim8Y34nc02GxAH8o551-e38E49o/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4639,17 +4639,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>VV-FRUKI01-001_Plano-VeV.md</t>
+          <t>VV-FRUKI01-001_Plano-VeV.docx</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pa1Kv-CVgiDKp6O15HsH2wS1Sj6w6rl2/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/15zwR3REjPc7plvrG3q3zeJKrpJCFi-BX/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4661,17 +4661,17 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>ADAP-FRUKI01-002_Registro-de-Adaptacao-PacoteFinal24.md</t>
+          <t>ADAP-FRUKI01-002_Registro-de-Adaptacao-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1gUQ1M-ZbVfLD2JDMMRy5dF-HwbZGqGT5/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1VMC6fRaDDblj024RkZaO_kRBPI5-AWb2/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4683,17 +4683,17 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-003_Ata-de-Aceite-Final.md</t>
+          <t>ATA-FRUKI01-003_Ata-de-Aceite-Final.docx</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1-aeqT0BAQN8q9aiSFDprKncgUGv35Tbw/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1JsjKR7P6hEv9Atyfx_kxA95bQG3uvdgI/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4705,17 +4705,17 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-004_Ata-Validacao-Sprint1-NaoAlocados.md</t>
+          <t>ATA-FRUKI01-004_Ata-Validacao-Sprint1-NaoAlocados.docx</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/16-FiineTnD7qs-K0efjHI8oveh067Pjb/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1-gn_pkcbdNRCSzLHi75m8fgkkw2ILrev/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4727,17 +4727,17 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-005_Ata-Validacao-Sprint2-RegraDeOuro.md</t>
+          <t>ATA-FRUKI01-005_Ata-Validacao-Sprint2-RegraDeOuro.docx</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pDeNymn8eEw1bg7neASDrMpjaHtKKF3m/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1gUsmWDj66IvWi1jdTBUwx1_jOV3qBMcr/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4749,17 +4749,17 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-006_Ata-Validacao-Sprint3-PDV.md</t>
+          <t>ATA-FRUKI01-006_Ata-Validacao-Sprint3-PDV.docx</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1tfZWSE26gCYWH3-cALxoyp66y9FEXp-R/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1ksGRCQp2uOce8XzQ6JUwXrY5Jm6gypth/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4771,17 +4771,17 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>ATA-FRUKI01-008_Ata-Kickoff-PacoteFinal24.md</t>
+          <t>ATA-FRUKI01-008_Ata-Kickoff-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1W-eIgotNpxwMJEQ3NO9CEQwVqcRKvOrq/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1AxV06s10xmWtcppFZdspU8YgwA0kK3zo/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4793,17 +4793,17 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>CR-FRUKI01-001_Solicitacao-de-Mudanca-RegraDeOuro.md</t>
+          <t>CR-FRUKI01-001_Solicitacao-de-Mudanca-RegraDeOuro.docx</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17fNk1TFIvfWh4C2O_pOGytMA5Gj9xgrr/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1lES6gbWkdIs_lGMYzw0Oinv_mhKMd9vv/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4815,17 +4815,17 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>ITP-FRUKI01-002_Estrategia-de-Integracao-PacoteFinal24.md</t>
+          <t>ITP-FRUKI01-002_Estrategia-de-Integracao-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1b7z0ytGUrMuvUxixgK9g_YtzJOIAFlaD/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1x6oQSghPGUoW4ALmte-BAWOesdL7LOej/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4837,17 +4837,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>PCP-FRUKI01-002_Documento-de-Design-PacoteFinal24.md</t>
+          <t>PCP-FRUKI01-002_Documento-de-Design-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17pKjVVEK0WOH8TP4tQrYY-1SEOD87_gn/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/12JPCWQwCPOeAqhPQlD2RhqgWlhF7RCi_/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4859,17 +4859,17 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>PLA-FRUKI01-002_Plano-de-Projeto-PacoteFinal24.md</t>
+          <t>PLA-FRUKI01-002_Plano-de-Projeto-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11HJg1b3_ko_YRr18_io0PeJKdqbBS6cz/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1X7aqRJ1cFWaFFDY2-PIZOr0LZY3aYPUs/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4881,17 +4881,17 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>RAC-FRUKI01-001_Relatorio-de-Acompanhamento.md</t>
+          <t>RAC-FRUKI01-001_Relatorio-de-Acompanhamento.docx</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1tJKc9cSokMjVl6ZUEGziBPortQ0w9vHs/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1wCqToBV70Od2cMUBDpQdRHprknhcf03v/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4903,17 +4903,17 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>RASTR-FRUKI01-002_Matriz-de-Rastreabilidade-PacoteFinal24.md</t>
+          <t>RASTR-FRUKI01-002_Matriz-de-Rastreabilidade-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1r2v_XLLzm37ySMynrN3AyLOGj1IHdnoW/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/16oO8wnQlq4M88T-Twa2PvUaJOT4PdNvN/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4925,17 +4925,17 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>REQ-FRUKI01-002_Documento-de-Requisitos-PacoteFinal24.md</t>
+          <t>REQ-FRUKI01-002_Documento-de-Requisitos-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Fb7MpfzPfNKM--4N94Tx49pUGvWBnKab/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1SLfbHTNWFb_AEyvA6NY1PZH2-yaCEQaQ/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4947,17 +4947,17 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>TAE-FRUKI01-002_Termo-de-Encerramento-PacoteFinal24.md</t>
+          <t>TAE-FRUKI01-002_Termo-de-Encerramento-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1qGo80blY7kzlFuXtUUCrkV6K427xB6SK/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1F3XBLU-UzqieEn0RGs0fVDI5DUrGsYIf/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4969,17 +4969,17 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>TAP-FRUKI01-002_Termo-de-Abertura-PacoteFinal24.md</t>
+          <t>TAP-FRUKI01-002_Termo-de-Abertura-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ngjegtxERo_jJObFfcYsUfNPw9yuC9PV/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1wHC3EjPGW68mXZ48j8CHpEgv0AYir6vt/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -4991,17 +4991,17 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>VV-FRUKI01-002_Plano-VeV-PacoteFinal24.md</t>
+          <t>VV-FRUKI01-002_Plano-VeV-PacoteFinal24.docx</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1WcBf_hl4Unrs6FsG4AHhcJ-NuAoEG1s5/view?usp=drivesdk</t>
+          <t>https://drive.google.com/file/d/1lvrkJPwro6_uYQ5o_5Lmy58Y0nv0mrwd/view?usp=drivesdk</t>
         </is>
       </c>
     </row>

</xml_diff>